<commit_message>
Add user guide to app
</commit_message>
<xml_diff>
--- a/data/country_baselines/Updated/country_baselines_summarised.xlsx
+++ b/data/country_baselines/Updated/country_baselines_summarised.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/country_baselines/Updated/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{BF29F2F3-1EB6-8046-A3DB-FBA4844A21DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{992ED7EE-D3C1-D945-892E-5ADFE210E698}"/>
+  <xr:revisionPtr revIDLastSave="6" documentId="8_{BF29F2F3-1EB6-8046-A3DB-FBA4844A21DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{97F56976-1DC5-6745-AB7B-49FEA0D446C9}"/>
   <bookViews>
-    <workbookView xWindow="340" yWindow="-17560" windowWidth="28800" windowHeight="17400" xr2:uid="{B6C5909B-EEA9-8C48-8CDE-83CD703FC43E}"/>
+    <workbookView xWindow="820" yWindow="-10700" windowWidth="28800" windowHeight="17400" xr2:uid="{B6C5909B-EEA9-8C48-8CDE-83CD703FC43E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -647,7 +647,7 @@
         <v>28</v>
       </c>
       <c r="B2" s="2">
-        <v>249541</v>
+        <v>334817</v>
       </c>
       <c r="C2">
         <v>0</v>

</xml_diff>

<commit_message>
Updated userguide and malawi data
</commit_message>
<xml_diff>
--- a/data/country_baselines/Updated/country_baselines_summarised.xlsx
+++ b/data/country_baselines/Updated/country_baselines_summarised.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/country_baselines/Updated/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="37" documentId="8_{BF29F2F3-1EB6-8046-A3DB-FBA4844A21DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A506EE72-A6F8-6C42-BF1A-1C532753F708}"/>
+  <xr:revisionPtr revIDLastSave="61" documentId="8_{BF29F2F3-1EB6-8046-A3DB-FBA4844A21DB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CCD2A679-0C38-2647-B118-D5134FCA8CF7}"/>
   <bookViews>
-    <workbookView xWindow="880" yWindow="-19400" windowWidth="28800" windowHeight="17400" xr2:uid="{B6C5909B-EEA9-8C48-8CDE-83CD703FC43E}"/>
+    <workbookView xWindow="2380" yWindow="600" windowWidth="28800" windowHeight="15820" xr2:uid="{B6C5909B-EEA9-8C48-8CDE-83CD703FC43E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -35,8 +35,35 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>tc={2310EEF3-F49B-1740-9531-F7745180ADE8}</author>
+    <author>tc={D2460033-F738-7142-809A-6A6DE4B461DC}</author>
+  </authors>
+  <commentList>
+    <comment ref="K4" authorId="0" shapeId="0" xr:uid="{2310EEF3-F49B-1740-9531-F7745180ADE8}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    Community-Based HIV Test in 2025</t>
+      </text>
+    </comment>
+    <comment ref="L4" authorId="1" shapeId="0" xr:uid="{D2460033-F738-7142-809A-6A6DE4B461DC}">
+      <text>
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
+    90% HIV Ascertainment in STI services</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t>prep_oral</t>
   </si>
@@ -126,6 +153,9 @@
   </si>
   <si>
     <t>Zambia</t>
+  </si>
+  <si>
+    <t>Malawi</t>
   </si>
 </sst>
 </file>
@@ -136,7 +166,7 @@
     <numFmt numFmtId="43" formatCode="_(* #,##0.00_);_(* \(#,##0.00\);_(* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_(* #,##0_);_(* \(#,##0\);_(* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -162,6 +192,18 @@
       <sz val="11"/>
       <color theme="1"/>
       <name val="Lucida Sans"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Tahoma"/>
       <family val="2"/>
     </font>
   </fonts>
@@ -230,7 +272,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
@@ -252,6 +294,9 @@
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="3" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -268,6 +313,12 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <person displayName="John Phiri" id="{5C421396-DDD7-7544-B72E-8164399E8CC5}" userId="S::jphiri@hivmw.org::153ac18e-b8b8-4307-ae1e-382ef26ad919" providerId="AD"/>
+</personList>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -585,12 +636,24 @@
 </a:theme>
 </file>
 
+<file path=xl/threadedComments/threadedComment1.xml><?xml version="1.0" encoding="utf-8"?>
+<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <threadedComment ref="K4" dT="2026-06-05T07:00:54.77" personId="{5C421396-DDD7-7544-B72E-8164399E8CC5}" id="{2310EEF3-F49B-1740-9531-F7745180ADE8}">
+    <text>Community-Based HIV Test in 2025</text>
+  </threadedComment>
+  <threadedComment ref="L4" dT="2026-06-05T07:06:08.87" personId="{5C421396-DDD7-7544-B72E-8164399E8CC5}" id="{D2460033-F738-7142-809A-6A6DE4B461DC}">
+    <text>90% HIV Ascertainment in STI services</text>
+  </threadedComment>
+</ThreadedComments>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E15A684A-C287-EF40-83C7-44769AE087D6}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E15A684A-C287-EF40-83C7-44769AE087D6}">
   <dimension ref="A1:AB29"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="3" max="3" width="15.1640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="17.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -833,7 +896,75 @@
       </c>
     </row>
     <row r="4" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A4" s="1"/>
+      <c r="A4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B4" s="11">
+        <v>58089</v>
+      </c>
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4" s="11">
+        <v>47890</v>
+      </c>
+      <c r="E4" s="11">
+        <v>139000000</v>
+      </c>
+      <c r="F4" s="12">
+        <v>32466</v>
+      </c>
+      <c r="G4" s="13">
+        <v>91</v>
+      </c>
+      <c r="H4" s="11">
+        <v>30762</v>
+      </c>
+      <c r="I4" s="11">
+        <v>3569803</v>
+      </c>
+      <c r="J4" s="11">
+        <v>129230</v>
+      </c>
+      <c r="K4" s="11">
+        <v>129013</v>
+      </c>
+      <c r="L4" s="11">
+        <v>513183</v>
+      </c>
+      <c r="M4" s="11">
+        <v>1741863</v>
+      </c>
+      <c r="N4" s="11">
+        <v>60432</v>
+      </c>
+      <c r="O4" s="13">
+        <v>88</v>
+      </c>
+      <c r="P4" s="13">
+        <v>96</v>
+      </c>
+      <c r="Q4" s="13">
+        <v>15</v>
+      </c>
+      <c r="R4">
+        <v>82</v>
+      </c>
+      <c r="S4">
+        <v>47</v>
+      </c>
+      <c r="T4">
+        <v>46</v>
+      </c>
+      <c r="U4">
+        <v>0</v>
+      </c>
+      <c r="V4">
+        <v>5</v>
+      </c>
+      <c r="AA4">
+        <v>57</v>
+      </c>
     </row>
     <row r="5" spans="1:28" x14ac:dyDescent="0.2">
       <c r="A5" s="1"/>
@@ -912,5 +1043,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
App dpeloy and wording
</commit_message>
<xml_diff>
--- a/data/country_baselines/Updated/country_baselines_summarised.xlsx
+++ b/data/country_baselines/Updated/country_baselines_summarised.xlsx
@@ -8,14 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/country_baselines/Updated/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="61" documentId="14_{78023D7A-79C9-BB4A-96DA-66D3AFB5E9C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CF33940D-B1A7-634B-AB05-2482FD5C76E5}"/>
+  <xr:revisionPtr revIDLastSave="64" documentId="14_{78023D7A-79C9-BB4A-96DA-66D3AFB5E9C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB8C1795-EFC0-DA46-9B56-828CF0ABCDAC}"/>
   <bookViews>
-    <workbookView xWindow="-32820" yWindow="3660" windowWidth="28800" windowHeight="15740" xr2:uid="{B6C5909B-EEA9-8C48-8CDE-83CD703FC43E}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15820" xr2:uid="{B6C5909B-EEA9-8C48-8CDE-83CD703FC43E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet1" sheetId="1" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -64,35 +63,8 @@
 </comments>
 </file>
 
-<file path=xl/comments2.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
-  <authors>
-    <author>tc={2310EEF3-F49B-1740-9531-F7745180ADE8}</author>
-    <author>tc={D2460033-F738-7142-809A-6A6DE4B461DC}</author>
-  </authors>
-  <commentList>
-    <comment ref="K4" authorId="0" shapeId="0" xr:uid="{2310EEF3-F49B-1740-9531-F7745180ADE8}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Community-Based HIV Test in 2025</t>
-      </text>
-    </comment>
-    <comment ref="L4" authorId="1" shapeId="0" xr:uid="{D2460033-F738-7142-809A-6A6DE4B461DC}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    90% HIV Ascertainment in STI services</t>
-      </text>
-    </comment>
-  </commentList>
-</comments>
-</file>
-
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="78" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
   <si>
     <t>prep_oral</t>
   </si>
@@ -736,17 +708,6 @@
 </ThreadedComments>
 </file>
 
-<file path=xl/threadedComments/threadedComment2.xml><?xml version="1.0" encoding="utf-8"?>
-<ThreadedComments xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <threadedComment ref="K4" dT="2026-06-05T07:00:54.77" personId="{5C421396-DDD7-7544-B72E-8164399E8CC5}" id="{2310EEF3-F49B-1740-9531-F7745180ADE8}">
-    <text>Community-Based HIV Test in 2025</text>
-  </threadedComment>
-  <threadedComment ref="L4" dT="2026-06-05T07:06:08.87" personId="{5C421396-DDD7-7544-B72E-8164399E8CC5}" id="{D2460033-F738-7142-809A-6A6DE4B461DC}">
-    <text>90% HIV Ascertainment in STI services</text>
-  </threadedComment>
-</ThreadedComments>
-</file>
-
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{42369831-8138-B640-8215-2EE7ACAC45E9}">
   <dimension ref="A1:AB29"/>
@@ -1385,406 +1346,13 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E15A684A-C287-EF40-83C7-44769AE087D6}">
-  <dimension ref="A1:AB29"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
-  <cols>
-    <col min="3" max="3" width="15.1640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="12.5" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="17.6640625" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="L1" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="M1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="P1" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="Q1" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="R1" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="S1" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="T1" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="V1" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="X1" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="Y1" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="Z1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AA1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="AB1" s="1" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="2" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A2" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B2" s="2">
-        <v>334817</v>
-      </c>
-      <c r="C2">
-        <v>0</v>
-      </c>
-      <c r="D2" s="2">
-        <v>147928</v>
-      </c>
-      <c r="E2">
-        <v>159303077</v>
-      </c>
-      <c r="H2">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2">
-        <v>11237387</v>
-      </c>
-      <c r="J2" s="2">
-        <v>630566</v>
-      </c>
-      <c r="K2" s="2">
-        <v>1064884</v>
-      </c>
-      <c r="L2" s="2">
-        <v>222182</v>
-      </c>
-      <c r="M2" s="3">
-        <v>0</v>
-      </c>
-      <c r="N2" s="2">
-        <v>1322885</v>
-      </c>
-      <c r="O2" s="4">
-        <v>90</v>
-      </c>
-      <c r="P2" s="4">
-        <v>95</v>
-      </c>
-      <c r="R2" s="5">
-        <v>67</v>
-      </c>
-      <c r="S2" s="5">
-        <v>37</v>
-      </c>
-      <c r="T2" s="5">
-        <v>40</v>
-      </c>
-      <c r="U2" s="5">
-        <v>0.1</v>
-      </c>
-      <c r="V2" s="5">
-        <v>2</v>
-      </c>
-      <c r="W2" s="5">
-        <v>50</v>
-      </c>
-      <c r="X2" s="5">
-        <v>85</v>
-      </c>
-      <c r="Y2" s="5">
-        <v>77</v>
-      </c>
-      <c r="Z2" s="5">
-        <v>80</v>
-      </c>
-      <c r="AA2" s="5">
-        <v>24</v>
-      </c>
-      <c r="AB2" s="5"/>
-    </row>
-    <row r="3" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="B3" s="6">
-        <v>133901</v>
-      </c>
-      <c r="C3" s="7">
-        <v>1624</v>
-      </c>
-      <c r="D3" s="6">
-        <v>274325</v>
-      </c>
-      <c r="F3" s="8">
-        <v>6454</v>
-      </c>
-      <c r="G3">
-        <v>74</v>
-      </c>
-      <c r="H3">
-        <v>0</v>
-      </c>
-      <c r="I3" s="9">
-        <v>3671497</v>
-      </c>
-      <c r="J3" s="9">
-        <v>291365</v>
-      </c>
-      <c r="K3" s="9">
-        <v>516869</v>
-      </c>
-      <c r="L3" s="10">
-        <v>0</v>
-      </c>
-      <c r="M3" s="10">
-        <v>0</v>
-      </c>
-      <c r="N3" s="10">
-        <v>0</v>
-      </c>
-      <c r="O3">
-        <v>76</v>
-      </c>
-      <c r="P3" s="10">
-        <v>93</v>
-      </c>
-      <c r="Q3" s="10">
-        <v>24</v>
-      </c>
-      <c r="R3">
-        <v>79</v>
-      </c>
-      <c r="S3">
-        <v>4</v>
-      </c>
-      <c r="T3">
-        <v>96</v>
-      </c>
-      <c r="U3">
-        <v>0</v>
-      </c>
-      <c r="V3">
-        <v>30</v>
-      </c>
-      <c r="W3">
-        <v>95</v>
-      </c>
-      <c r="X3">
-        <v>95</v>
-      </c>
-      <c r="AA3">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A4" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" s="11">
-        <v>58089</v>
-      </c>
-      <c r="C4">
-        <v>0</v>
-      </c>
-      <c r="D4" s="11">
-        <v>47890</v>
-      </c>
-      <c r="E4" s="11">
-        <v>139000000</v>
-      </c>
-      <c r="F4" s="12">
-        <v>32466</v>
-      </c>
-      <c r="G4" s="13">
-        <v>91</v>
-      </c>
-      <c r="H4" s="11">
-        <v>30762</v>
-      </c>
-      <c r="I4" s="11">
-        <v>3569803</v>
-      </c>
-      <c r="J4" s="11">
-        <v>129230</v>
-      </c>
-      <c r="K4" s="11">
-        <v>129013</v>
-      </c>
-      <c r="L4" s="11">
-        <v>513183</v>
-      </c>
-      <c r="M4" s="11">
-        <v>1741863</v>
-      </c>
-      <c r="N4" s="11">
-        <v>60432</v>
-      </c>
-      <c r="O4" s="13">
-        <v>88</v>
-      </c>
-      <c r="P4" s="13">
-        <v>96</v>
-      </c>
-      <c r="Q4" s="13">
-        <v>15</v>
-      </c>
-      <c r="R4">
-        <v>82</v>
-      </c>
-      <c r="S4">
-        <v>47</v>
-      </c>
-      <c r="T4">
-        <v>46</v>
-      </c>
-      <c r="U4">
-        <v>0</v>
-      </c>
-      <c r="V4">
-        <v>5</v>
-      </c>
-      <c r="AA4">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A5" s="1"/>
-    </row>
-    <row r="6" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A6" s="1"/>
-    </row>
-    <row r="7" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A7" s="1"/>
-    </row>
-    <row r="8" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A8" s="1"/>
-    </row>
-    <row r="9" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A9" s="1"/>
-    </row>
-    <row r="10" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A10" s="1"/>
-    </row>
-    <row r="11" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A11" s="1"/>
-    </row>
-    <row r="12" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A12" s="1"/>
-    </row>
-    <row r="13" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A13" s="1"/>
-    </row>
-    <row r="14" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A14" s="1"/>
-    </row>
-    <row r="15" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A15" s="1"/>
-    </row>
-    <row r="16" spans="1:28" x14ac:dyDescent="0.2">
-      <c r="A16" s="1"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="1"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="1"/>
-    </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A19" s="1"/>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="1"/>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="1"/>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" s="1"/>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" s="1"/>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" s="1"/>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" s="1"/>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="1"/>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" s="1"/>
-    </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A28" s="1"/>
-    </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" s="1"/>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{290418B9-1F0F-1140-BB8B-34C4D210D63F}">
   <dimension ref="A1:C6"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="29.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="5.1640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A1" t="s">

</xml_diff>

<commit_message>
Updates pre - slowness changes
</commit_message>
<xml_diff>
--- a/data/country_baselines/Updated/country_baselines_summarised.xlsx
+++ b/data/country_baselines/Updated/country_baselines_summarised.xlsx
@@ -8,13 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2ae90f5cbd0fd171/AMC/HIV Prioritization tool/HIV_prioritization_tool/data/country_baselines/Updated/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="64" documentId="14_{78023D7A-79C9-BB4A-96DA-66D3AFB5E9C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{AB8C1795-EFC0-DA46-9B56-828CF0ABCDAC}"/>
+  <xr:revisionPtr revIDLastSave="79" documentId="14_{78023D7A-79C9-BB4A-96DA-66D3AFB5E9C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5C572DB0-F928-534D-8DF4-0652EBE0DF45}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="28800" windowHeight="15820" xr2:uid="{B6C5909B-EEA9-8C48-8CDE-83CD703FC43E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId2"/>
+    <sheet name="SA data" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -64,7 +64,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="51">
   <si>
     <t>prep_oral</t>
   </si>
@@ -199,6 +199,24 @@
   </si>
   <si>
     <t>https://www.differentiatedservicedelivery.org/wp-content/uploads/NDOH-Prevention-Treatment-Care-and-Support-Priorities-_-Gates-Foundation-Partners-Meeting-11-12-Feb-2516.pdf</t>
+  </si>
+  <si>
+    <t>https://hst-assets-s3.s3.eu-north-1.amazonaws.com/publications/District-Health-Barometer-2024_2025.pdf</t>
+  </si>
+  <si>
+    <t>oral prep</t>
+  </si>
+  <si>
+    <t>https://www.spotlightnsp.co.za/2026/05/15/sas-arv-programme-hardly-grew-in-2025-according-to-latest-estimates/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">vmmc </t>
+  </si>
+  <si>
+    <t>~290000</t>
+  </si>
+  <si>
+    <t>Thembisa 2025. https://www.spotlightnsp.co.za/hiv-dashboard/</t>
   </si>
 </sst>
 </file>
@@ -1082,6 +1100,15 @@
       <c r="A6" s="1" t="s">
         <v>32</v>
       </c>
+      <c r="B6">
+        <v>580000</v>
+      </c>
+      <c r="D6">
+        <v>290000</v>
+      </c>
+      <c r="E6">
+        <v>685663529</v>
+      </c>
       <c r="O6">
         <v>73</v>
       </c>
@@ -1347,11 +1374,11 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{290418B9-1F0F-1140-BB8B-34C4D210D63F}">
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="29.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="5.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.2">
@@ -1414,6 +1441,39 @@
         <v>44</v>
       </c>
     </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" t="s">
+        <v>3</v>
+      </c>
+      <c r="B7">
+        <v>685663529</v>
+      </c>
+      <c r="C7" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8">
+        <v>580000</v>
+      </c>
+      <c r="C8" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B9" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>